<commit_message>
Main Web 18 Sep v2
</commit_message>
<xml_diff>
--- a/AtchisonRegime/assetsHTML/Atchison/SAAWeightsandRanges.xlsx
+++ b/AtchisonRegime/assetsHTML/Atchison/SAAWeightsandRanges.xlsx
@@ -1310,8 +1310,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005C6577D0C3AE724BBB504F46D5A19401" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="25845a2805ffec61273570ee8952a967">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="df76e320-99cb-4a11-b59f-8bf32867ab70" xmlns:ns3="c0789f30-979e-497b-8344-faefb3987540" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7888a8b67094cd90eeeebcd3ec37a641" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005C6577D0C3AE724BBB504F46D5A19401" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="17afb16e0fbe716d3dcf2481b32b5550">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="df76e320-99cb-4a11-b59f-8bf32867ab70" xmlns:ns3="c0789f30-979e-497b-8344-faefb3987540" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f6d0bb8d4e6a5d6b988ea2ed2503dbb5" ns2:_="" ns3:_="">
     <xsd:import namespace="df76e320-99cb-4a11-b59f-8bf32867ab70"/>
     <xsd:import namespace="c0789f30-979e-497b-8344-faefb3987540"/>
     <xsd:element name="properties">
@@ -1573,23 +1573,19 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="c0789f30-979e-497b-8344-faefb3987540" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="df76e320-99cb-4a11-b59f-8bf32867ab70">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{43767ECD-B03D-4046-9587-8ED06C51B473}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="df76e320-99cb-4a11-b59f-8bf32867ab70"/>
-    <ds:schemaRef ds:uri="c0789f30-979e-497b-8344-faefb3987540"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C38E378B-BE20-48B6-AC9F-11D889E074B8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1598,4 +1594,8 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A0B2283-E079-47A3-9A7D-0DFDB12ACCDE}"/>
 </file>
</xml_diff>